<commit_message>
Updated RAD Test Cases for Header and CF Changes plus other RAD updates
</commit_message>
<xml_diff>
--- a/KatalonData/RADTestData/BeforePayments.xlsx
+++ b/KatalonData/RADTestData/BeforePayments.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent>
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\t465179\Documents\git\VPS-Katalon\VPS-Katalon\KatalonData\RADTestData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr documentId="13_ncr:1_{D3B34142-0BD7-480B-8464-85977A0636C2}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
+  <xr:revisionPtr documentId="13_ncr:1_{A55B5BD7-60D1-4D2D-89E1-6A1B1ADDA73D}" revIDLastSave="0" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47"/>
   <bookViews>
-    <workbookView activeTab="3" windowHeight="15675" windowWidth="28995" xWindow="14303" xr2:uid="{D99FAB39-5CE6-4AA4-B9C6-99B1EFA0654E}" yWindow="-2010"/>
+    <workbookView activeTab="3" windowHeight="15675" windowWidth="28996" xWindow="-98" xr2:uid="{D99FAB39-5CE6-4AA4-B9C6-99B1EFA0654E}" yWindow="-98"/>
   </bookViews>
   <sheets>
     <sheet name="Estimated" r:id="rId1" sheetId="1"/>
@@ -46,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="897" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1354" uniqueCount="330">
   <si>
     <t>Result</t>
   </si>
@@ -423,313 +423,619 @@
     <t>Incorrect App ID</t>
   </si>
   <si>
-    <t>Mon Oct 13 20:52:40 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 20:53:24 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 20:54:06 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 20:54:48 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 20:55:28 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 20:56:08 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 20:56:48 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 20:57:27 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 20:58:06 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 20:58:47 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:00:09 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:00:49 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:01:28 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:13:37 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:14:20 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:15:01 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:15:55 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:16:41 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:17:23 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:18:51 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:19:39 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:20:18 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:21:01 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:21:56 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:22:35 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:24:14 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:24:54 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:25:49 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:26:28 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:27:20 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:28:00 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:28:40 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:33:44 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:34:37 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:35:21 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:37:05 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:38:03 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:38:42 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:40:45 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:41:24 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:42:12 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:42:54 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:43:57 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:44:48 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:45:34 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:46:14 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:46:55 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:47:43 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:49:42 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:50:42 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:51:30 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:52:10 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:52:53 EDT 2025</t>
-  </si>
-  <si>
-    <t>Mon Oct 13 21:58:51 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 14:57:28 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 14:58:10 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 14:58:48 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 14:59:27 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 15:00:07 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 15:03:07 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 15:03:55 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 15:04:38 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 15:05:23 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 15:06:07 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 22:16:58 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 22:17:42 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 22:18:20 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 22:19:01 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 22:19:39 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 22:20:33 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 22:26:20 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 22:27:45 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Oct 14 22:29:08 EDT 2025</t>
-  </si>
-  <si>
-    <t>Tue Nov 04 15:50:50 EST 2025</t>
-  </si>
-  <si>
-    <t>Tue Nov 04 15:57:52 EST 2025</t>
-  </si>
-  <si>
-    <t>Tue Nov 04 15:58:39 EST 2025</t>
-  </si>
-  <si>
-    <t>Tue Nov 04 16:25:09 EST 2025</t>
-  </si>
-  <si>
     <t>Fail</t>
   </si>
   <si>
-    <t>Wed Nov 05 16:47:11 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 16:48:08 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 16:49:03 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 16:49:59 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 16:50:54 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 16:51:50 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 17:02:29 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 17:07:52 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 17:49:09 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 17:50:04 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 18:09:34 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 18:18:08 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 20:13:59 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 20:14:56 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 20:15:53 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 20:16:50 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 20:17:51 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 20:18:55 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 20:33:56 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 20:51:39 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 20:57:58 EST 2025</t>
-  </si>
-  <si>
-    <t>Wed Nov 05 21:04:23 EST 2025</t>
-  </si>
-  <si>
     <t>This is in QA and Demo but not in Production</t>
   </si>
   <si>
+    <t>2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:27:17 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:28:05 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:28:50 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:29:34 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:30:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:31:02 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:31:47 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:32:33 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:33:21 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:34:10 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:34:58 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:35:43 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:36:29 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:37:16 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:38:03 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:38:51 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:39:37 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:40:20 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:41:04 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:41:48 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:42:32 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:43:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:44:02 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:44:44 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:45:29 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:46:13 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:47:12 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:47:56 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:48:39 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:49:23 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:50:09 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:50:53 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:51:36 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:52:20 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:53:04 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:53:47 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:54:30 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:55:15 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:55:58 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:56:42 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:57:26 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:58:11 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:58:53 EDT 2026</t>
+  </si>
+  <si>
+    <t>Thu May 28 23:59:37 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:00:24 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:01:08 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:01:52 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:02:36 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:03:21 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:04:07 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:04:51 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:05:34 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:06:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:07:02 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:07:46 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:08:31 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:09:14 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:09:57 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:10:41 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:11:31 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:12:15 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:12:58 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:13:43 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:14:27 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:15:11 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:16:00 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:16:43 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:17:27 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:18:11 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:18:54 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:19:37 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:20:21 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:21:05 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:21:49 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:22:33 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:23:17 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:24:02 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:24:45 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:25:29 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:26:13 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:26:57 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:27:40 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:28:25 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:29:09 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:29:52 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:30:51 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:31:34 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:32:33 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:33:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:34:21 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:35:07 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:35:52 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:36:38 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:37:25 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:38:10 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:38:56 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:39:47 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:40:38 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:41:29 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 00:42:21 EDT 2026</t>
+  </si>
+  <si>
     <t/>
   </si>
   <si>
-    <t>Thu Nov 27 16:52:17 EST 2025</t>
+    <t>Fri May 29 11:16:53 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:05:10 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:06:13 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:07:13 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:08:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:09:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:10:17 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:11:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:12:46 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:13:54 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:15:03 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:16:11 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:17:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:18:26 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:19:34 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:20:41 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:21:49 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:22:58 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:24:06 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:25:19 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:26:28 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:27:36 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:28:43 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:29:55 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:31:05 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:32:12 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:33:50 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:35:27 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:36:36 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:37:47 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:38:59 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:40:09 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:41:17 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:42:25 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:43:33 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:44:40 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:45:49 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:46:56 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:48:04 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:49:12 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:50:21 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:51:30 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:52:37 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:53:45 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:54:54 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:56:02 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:57:10 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:58:23 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 19:59:31 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:00:40 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:01:47 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:02:56 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:04:04 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:05:15 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:06:23 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:07:32 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:08:41 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:09:49 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:10:58 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:12:07 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:13:15 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:14:24 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:15:33 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:16:41 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:17:49 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:18:58 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:20:07 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:21:15 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:22:24 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:23:33 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:24:42 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:25:49 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:26:59 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:28:07 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:29:15 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:30:25 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:31:34 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:32:43 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:33:51 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:34:59 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:36:08 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:37:16 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:38:26 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:39:35 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:40:44 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:42:20 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:43:57 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:45:35 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:47:12 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:48:54 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:50:31 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:51:39 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:52:47 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:53:54 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:55:01 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:56:09 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:57:18 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:58:33 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 20:59:45 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 21:00:59 EDT 2026</t>
+  </si>
+  <si>
+    <t>Fri May 29 21:02:11 EDT 2026</t>
   </si>
 </sst>
 </file>
@@ -1106,23 +1412,23 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19BDCA51-7A9D-4BB2-A660-F3BEEC814D67}">
-  <dimension ref="A1:K7"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <dimension ref="A1:K8"/>
+  <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" style="1" width="9.1796875" collapsed="true"/>
-    <col min="2" max="2" customWidth="true" style="1" width="32.1796875" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="14.54296875" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" style="1" width="44.54296875" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="35.54296875" collapsed="true"/>
-    <col min="6" max="6" customWidth="true" style="1" width="15.26953125" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" style="1" width="17.26953125" collapsed="true"/>
-    <col min="8" max="8" customWidth="true" style="1" width="19.54296875" collapsed="true"/>
-    <col min="9" max="9" style="1" width="9.1796875" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" style="1" width="18.453125" collapsed="true"/>
-    <col min="11" max="16384" style="1" width="9.1796875" collapsed="true"/>
+    <col min="1" max="1" style="1" width="9.19921875" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" style="1" width="32.19921875" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="1" width="14.53125" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" style="1" width="44.53125" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" style="1" width="35.53125" collapsed="true"/>
+    <col min="6" max="6" customWidth="true" style="1" width="15.265625" collapsed="true"/>
+    <col min="7" max="7" customWidth="true" style="1" width="17.265625" collapsed="true"/>
+    <col min="8" max="8" customWidth="true" style="1" width="19.53125" collapsed="true"/>
+    <col min="9" max="9" style="1" width="9.19921875" collapsed="true"/>
+    <col min="10" max="10" customWidth="true" style="1" width="18.46484375" collapsed="true"/>
+    <col min="11" max="16384" style="1" width="9.19921875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1154,12 +1460,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>32</v>
@@ -1171,7 +1477,7 @@
         <v>8</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>19</v>
@@ -1183,12 +1489,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>200</v>
+        <v>231</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>32</v>
@@ -1200,7 +1506,7 @@
         <v>9</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>20</v>
@@ -1212,12 +1518,12 @@
         <v>51</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>198</v>
+        <v>232</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>32</v>
@@ -1229,7 +1535,7 @@
         <v>10</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>21</v>
@@ -1244,12 +1550,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>125</v>
+        <v>233</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>32</v>
@@ -1261,7 +1567,7 @@
         <v>11</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>22</v>
@@ -1276,12 +1582,12 @@
         <v>51</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>126</v>
+        <v>234</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>32</v>
@@ -1293,7 +1599,7 @@
         <v>12</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>23</v>
@@ -1308,12 +1614,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>127</v>
+        <v>235</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>32</v>
@@ -1325,7 +1631,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="G7" s="1" t="s">
         <v>24</v>
@@ -1338,6 +1644,29 @@
       </c>
       <c r="J7" s="1" t="s">
         <v>52</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
+      <c r="A8" t="s">
+        <v>125</v>
+      </c>
+      <c r="B8" t="s">
+        <v>236</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>102</v>
       </c>
     </row>
   </sheetData>
@@ -1353,21 +1682,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FAB49CF7-E4D4-4F06-BD88-EA9191F7BC6F}">
   <dimension ref="A1:K21"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" customWidth="true" style="1" width="14.54296875" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="27.26953125" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="12.6328125" collapsed="true"/>
+    <col min="1" max="1" customWidth="true" style="1" width="14.53125" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="27.265625" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="1" width="12.59765625" collapsed="true"/>
     <col min="4" max="4" customWidth="true" style="1" width="52.0" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="32.453125" collapsed="true"/>
-    <col min="6" max="7" style="1" width="9.1796875" collapsed="true"/>
-    <col min="8" max="8" customWidth="true" style="1" width="16.26953125" collapsed="true"/>
-    <col min="9" max="9" style="1" width="9.1796875" collapsed="true"/>
-    <col min="10" max="10" customWidth="true" style="1" width="43.36328125" collapsed="true"/>
-    <col min="11" max="16384" style="1" width="9.1796875" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" style="1" width="32.46484375" collapsed="true"/>
+    <col min="6" max="7" style="1" width="9.19921875" collapsed="true"/>
+    <col min="8" max="8" customWidth="true" style="1" width="16.265625" collapsed="true"/>
+    <col min="9" max="9" style="1" width="9.19921875" collapsed="true"/>
+    <col min="10" max="10" customWidth="true" style="1" width="43.33203125" collapsed="true"/>
+    <col min="11" max="16384" style="1" width="9.19921875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1399,12 +1728,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>128</v>
+        <v>237</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>32</v>
@@ -1422,12 +1751,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>129</v>
+        <v>238</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>32</v>
@@ -1445,12 +1774,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>130</v>
+        <v>239</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>32</v>
@@ -1468,12 +1797,12 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>131</v>
+        <v>240</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>32</v>
@@ -1494,12 +1823,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>132</v>
+        <v>241</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>32</v>
@@ -1520,12 +1849,12 @@
         <v>52</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>133</v>
+        <v>242</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>32</v>
@@ -1543,12 +1872,12 @@
         <v>63</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>134</v>
+        <v>243</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>32</v>
@@ -1566,12 +1895,12 @@
         <v>64</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>221</v>
+        <v>244</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>32</v>
@@ -1589,12 +1918,12 @@
         <v>65</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>135</v>
+        <v>245</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>32</v>
@@ -1612,12 +1941,12 @@
         <v>66</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>35</v>
       </c>
       <c r="B11" t="s">
-        <v>136</v>
+        <v>246</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>32</v>
@@ -1635,12 +1964,12 @@
         <v>67</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>35</v>
       </c>
       <c r="B12" t="s">
-        <v>137</v>
+        <v>247</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>32</v>
@@ -1658,12 +1987,12 @@
         <v>68</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>203</v>
+        <v>248</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>32</v>
@@ -1681,12 +2010,12 @@
         <v>69</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>204</v>
+        <v>249</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>32</v>
@@ -1704,12 +2033,12 @@
         <v>70</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>205</v>
+        <v>250</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>32</v>
@@ -1724,12 +2053,12 @@
         <v>71</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>206</v>
+        <v>251</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>32</v>
@@ -1750,12 +2079,12 @@
         <v>72</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>207</v>
+        <v>252</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>32</v>
@@ -1773,12 +2102,12 @@
         <v>73</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>208</v>
+        <v>253</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>32</v>
@@ -1796,7 +2125,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>35</v>
       </c>
@@ -1819,15 +2148,15 @@
         <v>75</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
-        <v>202</v>
+        <v>125</v>
       </c>
       <c r="B20" t="s">
-        <v>211</v>
+        <v>254</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>111</v>
@@ -1836,18 +2165,18 @@
         <v>115</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="21" spans="1:10" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
-        <v>202</v>
+        <v>125</v>
       </c>
       <c r="B21" t="s">
-        <v>212</v>
+        <v>255</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>111</v>
@@ -1859,7 +2188,7 @@
         <v>32</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>225</v>
+        <v>126</v>
       </c>
     </row>
   </sheetData>
@@ -1873,20 +2202,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A22222EF-2A37-441E-9CE4-90FD36DC8DDC}">
   <dimension ref="A1:J7"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" style="1" width="9.1796875" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="27.26953125" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="19.1796875" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" style="1" width="24.453125" collapsed="true"/>
+    <col min="1" max="1" style="1" width="9.19921875" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="27.265625" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="1" width="19.19921875" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" style="1" width="24.46484375" collapsed="true"/>
     <col min="5" max="5" bestFit="true" customWidth="true" style="1" width="27.0" collapsed="true"/>
-    <col min="6" max="6" style="1" width="9.1796875" collapsed="true"/>
+    <col min="6" max="6" style="1" width="9.19921875" collapsed="true"/>
     <col min="7" max="7" customWidth="true" style="1" width="17.0" collapsed="true"/>
-    <col min="8" max="8" customWidth="true" style="1" width="16.26953125" collapsed="true"/>
-    <col min="9" max="16384" style="1" width="9.1796875" collapsed="true"/>
+    <col min="8" max="8" customWidth="true" style="1" width="16.265625" collapsed="true"/>
+    <col min="9" max="16384" style="1" width="9.19921875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1915,12 +2244,12 @@
         <v>104</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>189</v>
+        <v>256</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>32</v>
@@ -1932,7 +2261,7 @@
         <v>8</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>22</v>
@@ -1941,12 +2270,12 @@
         <v>105</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>190</v>
+        <v>257</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>32</v>
@@ -1958,18 +2287,18 @@
         <v>9</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="I3" s="1" t="s">
         <v>106</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>191</v>
+        <v>258</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>32</v>
@@ -1981,7 +2310,7 @@
         <v>10</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="H4" s="1" t="s">
         <v>32</v>
@@ -1990,12 +2319,12 @@
         <v>107</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>192</v>
+        <v>259</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>32</v>
@@ -2007,7 +2336,7 @@
         <v>11</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="H5" s="1" t="s">
         <v>32</v>
@@ -2016,12 +2345,12 @@
         <v>108</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>193</v>
+        <v>260</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>32</v>
@@ -2033,7 +2362,7 @@
         <v>12</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>32</v>
@@ -2042,12 +2371,12 @@
         <v>109</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>194</v>
+        <v>261</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>32</v>
@@ -2059,7 +2388,7 @@
         <v>13</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="H7" s="1" t="s">
         <v>32</v>
@@ -2080,21 +2409,21 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E3B7105E-5E71-456F-8D2A-C4C503B29111}">
   <dimension ref="A1:M61"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" style="1" width="9.1796875" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="27.1796875" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="12.7265625" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" style="1" width="31.7265625" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="41.26953125" collapsed="true"/>
-    <col min="6" max="6" style="1" width="9.1796875" collapsed="true"/>
-    <col min="7" max="10" customWidth="true" style="1" width="19.81640625" collapsed="true"/>
-    <col min="11" max="11" style="1" width="9.1796875" collapsed="true"/>
-    <col min="12" max="12" customWidth="true" style="1" width="43.1796875" collapsed="true"/>
-    <col min="13" max="16384" style="1" width="9.1796875" collapsed="true"/>
+    <col min="1" max="1" style="1" width="9.19921875" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="27.19921875" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="1" width="12.73046875" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" style="1" width="31.73046875" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" style="1" width="41.265625" collapsed="true"/>
+    <col min="6" max="6" style="1" width="9.19921875" collapsed="true"/>
+    <col min="7" max="10" customWidth="true" style="1" width="19.796875" collapsed="true"/>
+    <col min="11" max="11" style="1" width="9.19921875" collapsed="true"/>
+    <col min="12" max="12" customWidth="true" style="1" width="43.19921875" collapsed="true"/>
+    <col min="13" max="16384" style="1" width="9.19921875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2132,12 +2461,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>209</v>
+        <v>262</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>32</v>
@@ -2148,19 +2477,19 @@
       <c r="E2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="1">
-        <v>2024</v>
+      <c r="F2" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="K2" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>201</v>
+        <v>263</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>32</v>
@@ -2171,8 +2500,8 @@
       <c r="E3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F3" s="1">
-        <v>2024</v>
+      <c r="F3" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>32</v>
@@ -2181,12 +2510,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>138</v>
+        <v>264</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>32</v>
@@ -2197,8 +2526,8 @@
       <c r="E4" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F4" s="1">
-        <v>2024</v>
+      <c r="F4" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>32</v>
@@ -2207,12 +2536,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>139</v>
+        <v>265</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>32</v>
@@ -2223,8 +2552,8 @@
       <c r="E5" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="1">
-        <v>2024</v>
+      <c r="F5" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>32</v>
@@ -2233,12 +2562,12 @@
         <v>79</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>140</v>
+        <v>266</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>32</v>
@@ -2249,8 +2578,8 @@
       <c r="E6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F6" s="1">
-        <v>2024</v>
+      <c r="F6" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>32</v>
@@ -2259,12 +2588,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>35</v>
       </c>
       <c r="B7" t="s">
-        <v>141</v>
+        <v>267</v>
       </c>
       <c r="C7" s="1" t="s">
         <v>32</v>
@@ -2275,19 +2604,19 @@
       <c r="E7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F7" s="1">
-        <v>2023</v>
+      <c r="F7" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>35</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>268</v>
       </c>
       <c r="C8" s="1" t="s">
         <v>32</v>
@@ -2298,8 +2627,8 @@
       <c r="E8" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F8" s="1">
-        <v>2023</v>
+      <c r="F8" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G8" s="1" t="s">
         <v>32</v>
@@ -2308,12 +2637,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>35</v>
       </c>
       <c r="B9" t="s">
-        <v>143</v>
+        <v>269</v>
       </c>
       <c r="C9" s="1" t="s">
         <v>32</v>
@@ -2324,8 +2653,8 @@
       <c r="E9" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F9" s="1">
-        <v>2023</v>
+      <c r="F9" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G9" s="1" t="s">
         <v>32</v>
@@ -2334,12 +2663,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B10" t="s">
-        <v>210</v>
+        <v>270</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>32</v>
@@ -2350,8 +2679,8 @@
       <c r="E10" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F10" s="1">
-        <v>2023</v>
+      <c r="F10" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G10" s="1" t="s">
         <v>32</v>
@@ -2360,12 +2689,12 @@
         <v>79</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>35</v>
       </c>
       <c r="B11" t="s">
-        <v>144</v>
+        <v>271</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>32</v>
@@ -2376,8 +2705,8 @@
       <c r="E11" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F11" s="1">
-        <v>2023</v>
+      <c r="F11" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G11" s="1" t="s">
         <v>32</v>
@@ -2386,12 +2715,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>35</v>
       </c>
       <c r="B12" t="s">
-        <v>145</v>
+        <v>272</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>32</v>
@@ -2402,19 +2731,19 @@
       <c r="E12" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="F12" s="1">
-        <v>2022</v>
+      <c r="F12" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="K12" s="1" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>35</v>
       </c>
       <c r="B13" t="s">
-        <v>146</v>
+        <v>273</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>32</v>
@@ -2425,8 +2754,8 @@
       <c r="E13" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F13" s="1">
-        <v>2022</v>
+      <c r="F13" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="G13" s="1" t="s">
         <v>32</v>
@@ -2435,12 +2764,12 @@
         <v>77</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>35</v>
       </c>
       <c r="B14" t="s">
-        <v>147</v>
+        <v>274</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>32</v>
@@ -2451,8 +2780,8 @@
       <c r="E14" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="F14" s="1">
-        <v>2022</v>
+      <c r="F14" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="G14" s="1" t="s">
         <v>32</v>
@@ -2461,12 +2790,12 @@
         <v>78</v>
       </c>
     </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>35</v>
       </c>
       <c r="B15" t="s">
-        <v>148</v>
+        <v>275</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>32</v>
@@ -2477,8 +2806,8 @@
       <c r="E15" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="F15" s="1">
-        <v>2022</v>
+      <c r="F15" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="G15" s="1" t="s">
         <v>32</v>
@@ -2487,12 +2816,12 @@
         <v>79</v>
       </c>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>35</v>
       </c>
       <c r="B16" t="s">
-        <v>149</v>
+        <v>276</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>32</v>
@@ -2503,8 +2832,8 @@
       <c r="E16" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="F16" s="1">
-        <v>2022</v>
+      <c r="F16" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="G16" s="1" t="s">
         <v>32</v>
@@ -2513,12 +2842,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="17" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B17" t="s">
-        <v>222</v>
+        <v>277</v>
       </c>
       <c r="C17" s="1" t="s">
         <v>32</v>
@@ -2529,8 +2858,8 @@
       <c r="E17" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F17" s="1">
-        <v>2025</v>
+      <c r="F17" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="H17" s="1" t="s">
         <v>32</v>
@@ -2542,12 +2871,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="18" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>35</v>
       </c>
       <c r="B18" t="s">
-        <v>150</v>
+        <v>278</v>
       </c>
       <c r="C18" s="1" t="s">
         <v>32</v>
@@ -2558,8 +2887,8 @@
       <c r="E18" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F18" s="1">
-        <v>2025</v>
+      <c r="F18" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="H18" s="1" t="s">
         <v>32</v>
@@ -2571,12 +2900,12 @@
         <v>82</v>
       </c>
     </row>
-    <row r="19" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>35</v>
       </c>
       <c r="B19" t="s">
-        <v>151</v>
+        <v>279</v>
       </c>
       <c r="C19" s="1" t="s">
         <v>32</v>
@@ -2587,8 +2916,8 @@
       <c r="E19" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F19" s="1">
-        <v>2025</v>
+      <c r="F19" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="H19" s="1" t="s">
         <v>32</v>
@@ -2600,12 +2929,12 @@
         <v>83</v>
       </c>
     </row>
-    <row r="20" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
         <v>35</v>
       </c>
       <c r="B20" t="s">
-        <v>152</v>
+        <v>280</v>
       </c>
       <c r="C20" s="1" t="s">
         <v>32</v>
@@ -2616,19 +2945,19 @@
       <c r="E20" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F20" s="1">
-        <v>2024</v>
+      <c r="F20" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="K20" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="21" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A21" t="s">
         <v>35</v>
       </c>
       <c r="B21" t="s">
-        <v>153</v>
+        <v>281</v>
       </c>
       <c r="C21" s="1" t="s">
         <v>32</v>
@@ -2639,8 +2968,8 @@
       <c r="E21" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F21" s="1">
-        <v>2025</v>
+      <c r="F21" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="I21" s="1" t="s">
         <v>98</v>
@@ -2652,12 +2981,12 @@
         <v>85</v>
       </c>
     </row>
-    <row r="22" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A22" t="s">
         <v>35</v>
       </c>
       <c r="B22" t="s">
-        <v>154</v>
+        <v>282</v>
       </c>
       <c r="C22" s="1" t="s">
         <v>32</v>
@@ -2668,8 +2997,8 @@
       <c r="E22" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F22" s="1">
-        <v>2025</v>
+      <c r="F22" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="H22" s="1" t="s">
         <v>32</v>
@@ -2681,12 +3010,12 @@
         <v>86</v>
       </c>
     </row>
-    <row r="23" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
         <v>35</v>
       </c>
       <c r="B23" t="s">
-        <v>155</v>
+        <v>283</v>
       </c>
       <c r="C23" s="1" t="s">
         <v>32</v>
@@ -2697,8 +3026,8 @@
       <c r="E23" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F23" s="1">
-        <v>2025</v>
+      <c r="F23" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="H23" s="1" t="s">
         <v>32</v>
@@ -2707,12 +3036,12 @@
         <v>87</v>
       </c>
     </row>
-    <row r="24" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A24" t="s">
         <v>35</v>
       </c>
       <c r="B24" t="s">
-        <v>156</v>
+        <v>284</v>
       </c>
       <c r="C24" s="1" t="s">
         <v>32</v>
@@ -2723,8 +3052,8 @@
       <c r="E24" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F24" s="1">
-        <v>2025</v>
+      <c r="F24" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="H24" s="1" t="s">
         <v>32</v>
@@ -2736,12 +3065,12 @@
         <v>88</v>
       </c>
     </row>
-    <row r="25" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A25" t="s">
         <v>35</v>
       </c>
       <c r="B25" t="s">
-        <v>195</v>
+        <v>285</v>
       </c>
       <c r="C25" s="1" t="s">
         <v>32</v>
@@ -2752,8 +3081,8 @@
       <c r="E25" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F25" s="1">
-        <v>2025</v>
+      <c r="F25" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="G25" s="1" t="s">
         <v>32</v>
@@ -2768,12 +3097,12 @@
         <v>89</v>
       </c>
     </row>
-    <row r="26" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A26" t="s">
         <v>35</v>
       </c>
       <c r="B26" t="s">
-        <v>196</v>
+        <v>286</v>
       </c>
       <c r="C26" s="1" t="s">
         <v>32</v>
@@ -2784,8 +3113,8 @@
       <c r="E26" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F26" s="1">
-        <v>2025</v>
+      <c r="F26" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="H26" s="1" t="s">
         <v>32</v>
@@ -2797,12 +3126,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="27" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A27" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B27" t="s">
-        <v>223</v>
+        <v>287</v>
       </c>
       <c r="C27" s="1" t="s">
         <v>32</v>
@@ -2813,8 +3142,8 @@
       <c r="E27" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F27" s="1">
-        <v>2025</v>
+      <c r="F27" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="G27" s="1" t="s">
         <v>32</v>
@@ -2826,12 +3155,12 @@
         <v>91</v>
       </c>
     </row>
-    <row r="28" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
         <v>35</v>
       </c>
       <c r="B28" t="s">
-        <v>197</v>
+        <v>288</v>
       </c>
       <c r="C28" s="1" t="s">
         <v>32</v>
@@ -2842,8 +3171,8 @@
       <c r="E28" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F28" s="1">
-        <v>2025</v>
+      <c r="F28" s="1" t="s">
+        <v>127</v>
       </c>
       <c r="H28" s="1" t="s">
         <v>32</v>
@@ -2858,12 +3187,12 @@
         <v>124</v>
       </c>
     </row>
-    <row r="29" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A29" t="s">
         <v>35</v>
       </c>
       <c r="B29" t="s">
-        <v>157</v>
+        <v>289</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>32</v>
@@ -2874,8 +3203,8 @@
       <c r="E29" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F29" s="1">
-        <v>2024</v>
+      <c r="F29" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="H29" s="1" t="s">
         <v>32</v>
@@ -2887,12 +3216,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="30" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A30" t="s">
         <v>35</v>
       </c>
       <c r="B30" t="s">
-        <v>158</v>
+        <v>290</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>32</v>
@@ -2904,7 +3233,7 @@
         <v>29</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="H30" s="1" t="s">
         <v>32</v>
@@ -2916,12 +3245,12 @@
         <v>82</v>
       </c>
     </row>
-    <row r="31" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A31" t="s">
         <v>35</v>
       </c>
       <c r="B31" t="s">
-        <v>159</v>
+        <v>291</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>32</v>
@@ -2932,8 +3261,8 @@
       <c r="E31" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F31" s="1">
-        <v>2024</v>
+      <c r="F31" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="H31" s="1" t="s">
         <v>32</v>
@@ -2945,12 +3274,12 @@
         <v>83</v>
       </c>
     </row>
-    <row r="32" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A32" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B32" t="s">
-        <v>213</v>
+        <v>292</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>32</v>
@@ -2961,19 +3290,19 @@
       <c r="E32" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F32" s="1">
-        <v>2023</v>
+      <c r="F32" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="K32" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="33" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
         <v>35</v>
       </c>
       <c r="B33" t="s">
-        <v>160</v>
+        <v>293</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>32</v>
@@ -2984,8 +3313,8 @@
       <c r="E33" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F33" s="1">
-        <v>2024</v>
+      <c r="F33" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="I33" s="1" t="s">
         <v>98</v>
@@ -2997,12 +3326,12 @@
         <v>85</v>
       </c>
     </row>
-    <row r="34" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A34" t="s">
         <v>35</v>
       </c>
       <c r="B34" t="s">
-        <v>161</v>
+        <v>294</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>32</v>
@@ -3013,8 +3342,8 @@
       <c r="E34" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F34" s="1">
-        <v>2024</v>
+      <c r="F34" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="H34" s="1" t="s">
         <v>32</v>
@@ -3026,12 +3355,12 @@
         <v>86</v>
       </c>
     </row>
-    <row r="35" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
         <v>35</v>
       </c>
       <c r="B35" t="s">
-        <v>162</v>
+        <v>295</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>32</v>
@@ -3042,8 +3371,8 @@
       <c r="E35" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F35" s="1">
-        <v>2024</v>
+      <c r="F35" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="H35" s="1" t="s">
         <v>32</v>
@@ -3052,12 +3381,12 @@
         <v>87</v>
       </c>
     </row>
-    <row r="36" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>224</v>
+        <v>296</v>
       </c>
       <c r="C36" s="1" t="s">
         <v>32</v>
@@ -3068,8 +3397,8 @@
       <c r="E36" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F36" s="1">
-        <v>2024</v>
+      <c r="F36" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="H36" s="1" t="s">
         <v>32</v>
@@ -3081,12 +3410,12 @@
         <v>88</v>
       </c>
     </row>
-    <row r="37" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
         <v>35</v>
       </c>
       <c r="B37" t="s">
-        <v>163</v>
+        <v>297</v>
       </c>
       <c r="C37" s="1" t="s">
         <v>32</v>
@@ -3097,8 +3426,8 @@
       <c r="E37" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F37" s="1">
-        <v>2024</v>
+      <c r="F37" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G37" s="1" t="s">
         <v>32</v>
@@ -3113,12 +3442,12 @@
         <v>89</v>
       </c>
     </row>
-    <row r="38" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
         <v>35</v>
       </c>
       <c r="B38" t="s">
-        <v>164</v>
+        <v>298</v>
       </c>
       <c r="C38" s="1" t="s">
         <v>32</v>
@@ -3129,8 +3458,8 @@
       <c r="E38" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F38" s="1">
-        <v>2024</v>
+      <c r="F38" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="H38" s="1" t="s">
         <v>32</v>
@@ -3142,12 +3471,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="39" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
         <v>35</v>
       </c>
       <c r="B39" t="s">
-        <v>165</v>
+        <v>299</v>
       </c>
       <c r="C39" s="1" t="s">
         <v>32</v>
@@ -3158,8 +3487,8 @@
       <c r="E39" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F39" s="1">
-        <v>2024</v>
+      <c r="F39" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="G39" s="1" t="s">
         <v>32</v>
@@ -3171,12 +3500,12 @@
         <v>91</v>
       </c>
     </row>
-    <row r="40" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A40" t="s">
         <v>35</v>
       </c>
       <c r="B40" t="s">
-        <v>166</v>
+        <v>300</v>
       </c>
       <c r="C40" s="1" t="s">
         <v>32</v>
@@ -3187,8 +3516,8 @@
       <c r="E40" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F40" s="1">
-        <v>2024</v>
+      <c r="F40" s="1" t="s">
+        <v>113</v>
       </c>
       <c r="H40" s="1" t="s">
         <v>32</v>
@@ -3203,12 +3532,12 @@
         <v>124</v>
       </c>
     </row>
-    <row r="41" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A41" t="s">
         <v>35</v>
       </c>
       <c r="B41" t="s">
-        <v>167</v>
+        <v>301</v>
       </c>
       <c r="C41" s="1" t="s">
         <v>32</v>
@@ -3219,8 +3548,8 @@
       <c r="E41" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="F41" s="1">
-        <v>2023</v>
+      <c r="F41" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="H41" s="1" t="s">
         <v>32</v>
@@ -3232,12 +3561,12 @@
         <v>81</v>
       </c>
     </row>
-    <row r="42" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A42" t="s">
         <v>35</v>
       </c>
       <c r="B42" t="s">
-        <v>168</v>
+        <v>302</v>
       </c>
       <c r="C42" s="1" t="s">
         <v>32</v>
@@ -3248,8 +3577,8 @@
       <c r="E42" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="F42" s="1">
-        <v>2023</v>
+      <c r="F42" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="H42" s="1" t="s">
         <v>32</v>
@@ -3261,12 +3590,12 @@
         <v>82</v>
       </c>
     </row>
-    <row r="43" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
         <v>35</v>
       </c>
       <c r="B43" t="s">
-        <v>169</v>
+        <v>303</v>
       </c>
       <c r="C43" s="1" t="s">
         <v>32</v>
@@ -3277,8 +3606,8 @@
       <c r="E43" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="F43" s="1">
-        <v>2023</v>
+      <c r="F43" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="H43" s="1" t="s">
         <v>32</v>
@@ -3290,12 +3619,12 @@
         <v>83</v>
       </c>
     </row>
-    <row r="44" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
         <v>35</v>
       </c>
       <c r="B44" t="s">
-        <v>170</v>
+        <v>304</v>
       </c>
       <c r="C44" s="1" t="s">
         <v>32</v>
@@ -3306,19 +3635,19 @@
       <c r="E44" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="F44" s="1">
-        <v>2022</v>
+      <c r="F44" s="1" t="s">
+        <v>18</v>
       </c>
       <c r="K44" s="1" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="45" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A45" t="s">
         <v>35</v>
       </c>
       <c r="B45" t="s">
-        <v>171</v>
+        <v>305</v>
       </c>
       <c r="C45" s="1" t="s">
         <v>32</v>
@@ -3329,8 +3658,8 @@
       <c r="E45" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F45" s="1">
-        <v>2023</v>
+      <c r="F45" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="I45" s="1" t="s">
         <v>98</v>
@@ -3342,12 +3671,12 @@
         <v>85</v>
       </c>
     </row>
-    <row r="46" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
         <v>35</v>
       </c>
       <c r="B46" t="s">
-        <v>172</v>
+        <v>306</v>
       </c>
       <c r="C46" s="1" t="s">
         <v>32</v>
@@ -3358,8 +3687,8 @@
       <c r="E46" s="1" t="s">
         <v>46</v>
       </c>
-      <c r="F46" s="1">
-        <v>2023</v>
+      <c r="F46" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="H46" s="1" t="s">
         <v>32</v>
@@ -3371,12 +3700,12 @@
         <v>86</v>
       </c>
     </row>
-    <row r="47" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A47" t="s">
-        <v>202</v>
+        <v>35</v>
       </c>
       <c r="B47" t="s">
-        <v>214</v>
+        <v>307</v>
       </c>
       <c r="C47" s="1" t="s">
         <v>32</v>
@@ -3387,8 +3716,8 @@
       <c r="E47" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="F47" s="1">
-        <v>2023</v>
+      <c r="F47" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="H47" s="1" t="s">
         <v>32</v>
@@ -3397,12 +3726,12 @@
         <v>87</v>
       </c>
     </row>
-    <row r="48" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A48" t="s">
         <v>35</v>
       </c>
       <c r="B48" t="s">
-        <v>173</v>
+        <v>308</v>
       </c>
       <c r="C48" s="1" t="s">
         <v>32</v>
@@ -3413,8 +3742,8 @@
       <c r="E48" s="1" t="s">
         <v>27</v>
       </c>
-      <c r="F48" s="1">
-        <v>2023</v>
+      <c r="F48" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="H48" s="1" t="s">
         <v>32</v>
@@ -3426,12 +3755,12 @@
         <v>88</v>
       </c>
     </row>
-    <row r="49" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A49" t="s">
         <v>35</v>
       </c>
       <c r="B49" t="s">
-        <v>174</v>
+        <v>309</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>32</v>
@@ -3442,8 +3771,8 @@
       <c r="E49" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="F49" s="1">
-        <v>2023</v>
+      <c r="F49" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G49" s="1" t="s">
         <v>32</v>
@@ -3458,12 +3787,12 @@
         <v>89</v>
       </c>
     </row>
-    <row r="50" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
         <v>35</v>
       </c>
       <c r="B50" t="s">
-        <v>175</v>
+        <v>310</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>32</v>
@@ -3474,8 +3803,8 @@
       <c r="E50" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="F50" s="1">
-        <v>2023</v>
+      <c r="F50" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="H50" s="1" t="s">
         <v>32</v>
@@ -3487,12 +3816,12 @@
         <v>90</v>
       </c>
     </row>
-    <row r="51" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
         <v>35</v>
       </c>
       <c r="B51" t="s">
-        <v>176</v>
+        <v>311</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>32</v>
@@ -3503,8 +3832,8 @@
       <c r="E51" s="1" t="s">
         <v>44</v>
       </c>
-      <c r="F51" s="1">
-        <v>2023</v>
+      <c r="F51" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="G51" s="1" t="s">
         <v>32</v>
@@ -3516,12 +3845,12 @@
         <v>91</v>
       </c>
     </row>
-    <row r="52" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
         <v>35</v>
       </c>
       <c r="B52" t="s">
-        <v>177</v>
+        <v>312</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>32</v>
@@ -3532,8 +3861,8 @@
       <c r="E52" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="F52" s="1">
-        <v>2023</v>
+      <c r="F52" s="1" t="s">
+        <v>37</v>
       </c>
       <c r="H52" s="1" t="s">
         <v>32</v>
@@ -3548,15 +3877,15 @@
         <v>124</v>
       </c>
     </row>
-    <row r="53" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A53" t="s">
-        <v>202</v>
+        <v>125</v>
       </c>
       <c r="B53" t="s">
-        <v>215</v>
+        <v>313</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D53" s="1" t="s">
         <v>16</v>
@@ -3565,21 +3894,21 @@
         <v>115</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="L53" s="1" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="54" spans="1:12" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="54" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A54" t="s">
-        <v>202</v>
+        <v>125</v>
       </c>
       <c r="B54" t="s">
-        <v>216</v>
+        <v>314</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D54" s="1" t="s">
         <v>16</v>
@@ -3588,16 +3917,16 @@
         <v>114</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="G54" s="1" t="s">
         <v>32</v>
       </c>
       <c r="L54" s="1" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="55" spans="1:12" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="55" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
         <v>35</v>
       </c>
@@ -3614,7 +3943,7 @@
         <v>45</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="G55" s="1" t="s">
         <v>32</v>
@@ -3623,15 +3952,15 @@
         <v>23</v>
       </c>
     </row>
-    <row r="56" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A56" t="s">
-        <v>202</v>
+        <v>125</v>
       </c>
       <c r="B56" t="s">
-        <v>217</v>
+        <v>315</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D56" s="1" t="s">
         <v>16</v>
@@ -3640,21 +3969,21 @@
         <v>115</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="L56" s="1" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="57" spans="1:12" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="57" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A57" t="s">
-        <v>202</v>
+        <v>125</v>
       </c>
       <c r="B57" t="s">
-        <v>218</v>
+        <v>316</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D57" s="1" t="s">
         <v>16</v>
@@ -3663,16 +3992,16 @@
         <v>114</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="G57" s="1" t="s">
         <v>32</v>
       </c>
       <c r="L57" s="1" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="58" spans="1:12" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="58" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A58" t="s">
         <v>35</v>
       </c>
@@ -3689,7 +4018,7 @@
         <v>45</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="G58" s="1" t="s">
         <v>32</v>
@@ -3698,15 +4027,15 @@
         <v>101</v>
       </c>
     </row>
-    <row r="59" spans="1:12" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
-        <v>202</v>
+        <v>125</v>
       </c>
       <c r="B59" t="s">
-        <v>219</v>
+        <v>317</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D59" s="1" t="s">
         <v>16</v>
@@ -3715,21 +4044,21 @@
         <v>115</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="L59" s="1" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="60" spans="1:12" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="60" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A60" t="s">
-        <v>202</v>
+        <v>125</v>
       </c>
       <c r="B60" t="s">
-        <v>220</v>
+        <v>318</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="D60" s="1" t="s">
         <v>16</v>
@@ -3738,16 +4067,16 @@
         <v>114</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="G60" s="1" t="s">
         <v>32</v>
       </c>
       <c r="L60" s="1" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="61" spans="1:12" x14ac:dyDescent="0.35">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="61" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A61" t="s">
         <v>35</v>
       </c>
@@ -3764,7 +4093,7 @@
         <v>45</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="G61" s="1" t="s">
         <v>32</v>
@@ -3786,17 +4115,17 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C48EC9F-E6C0-40A2-877C-8FE515BAA791}">
   <dimension ref="A1:G7"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" style="1" width="9.1796875" collapsed="true"/>
-    <col min="2" max="2" customWidth="true" style="1" width="22.453125" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="26.26953125" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" style="1" width="50.81640625" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="46.26953125" collapsed="true"/>
-    <col min="6" max="16384" style="1" width="9.1796875" collapsed="true"/>
+    <col min="1" max="1" style="1" width="9.19921875" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" style="1" width="22.46484375" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="1" width="26.265625" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" style="1" width="50.796875" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" style="1" width="46.265625" collapsed="true"/>
+    <col min="6" max="16384" style="1" width="9.19921875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3816,7 +4145,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="C2" s="1" t="s">
         <v>32</v>
       </c>
@@ -3830,7 +4159,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="C3" s="1" t="s">
         <v>32</v>
       </c>
@@ -3841,7 +4170,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="C4" s="1" t="s">
         <v>36</v>
       </c>
@@ -3855,7 +4184,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="C5" s="1" t="s">
         <v>32</v>
       </c>
@@ -3869,7 +4198,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="C6" s="1" t="s">
         <v>32</v>
       </c>
@@ -3883,7 +4212,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="C7" s="1" t="s">
         <v>32</v>
       </c>
@@ -3908,19 +4237,19 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AE13C096-3F8A-4B4D-A3EE-3415763F7F13}">
   <dimension ref="A1:I9"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" style="1" width="9.1796875" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="27.54296875" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="15.1796875" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" style="1" width="50.81640625" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="46.26953125" collapsed="true"/>
-    <col min="6" max="7" style="1" width="9.1796875" collapsed="true"/>
-    <col min="8" max="8" customWidth="true" style="1" width="23.453125" collapsed="true"/>
-    <col min="9" max="16384" style="1" width="9.1796875" collapsed="true"/>
+    <col min="1" max="1" style="1" width="9.19921875" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="27.53125" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="1" width="15.19921875" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" style="1" width="50.796875" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" style="1" width="46.265625" collapsed="true"/>
+    <col min="6" max="7" style="1" width="9.19921875" collapsed="true"/>
+    <col min="8" max="8" customWidth="true" style="1" width="23.46484375" collapsed="true"/>
+    <col min="9" max="16384" style="1" width="9.19921875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -3946,12 +4275,12 @@
         <v>50</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>179</v>
+        <v>320</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>32</v>
@@ -3963,18 +4292,18 @@
         <v>17</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>180</v>
+        <v>321</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>32</v>
@@ -3986,18 +4315,18 @@
         <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>181</v>
+        <v>322</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>32</v>
@@ -4009,18 +4338,18 @@
         <v>17</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>182</v>
+        <v>323</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>32</v>
@@ -4032,18 +4361,18 @@
         <v>17</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>183</v>
+        <v>324</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>32</v>
@@ -4055,13 +4384,13 @@
         <v>17</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>35</v>
       </c>
@@ -4081,7 +4410,7 @@
         <v>113</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>35</v>
       </c>
@@ -4101,7 +4430,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>35</v>
       </c>
@@ -4129,19 +4458,19 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7A156AB6-80FF-4E48-B399-7CA373BDFD42}">
   <dimension ref="A1:H6"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" style="1" width="9.1796875" collapsed="true"/>
-    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="26.453125" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="16.26953125" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" style="1" width="50.81640625" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="46.26953125" collapsed="true"/>
-    <col min="6" max="6" style="1" width="9.1796875" collapsed="true"/>
-    <col min="7" max="7" customWidth="true" style="1" width="14.1796875" collapsed="true"/>
-    <col min="8" max="16384" style="1" width="9.1796875" collapsed="true"/>
+    <col min="1" max="1" style="1" width="9.19921875" collapsed="true"/>
+    <col min="2" max="2" bestFit="true" customWidth="true" style="1" width="26.46484375" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="1" width="16.265625" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" style="1" width="50.796875" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" style="1" width="46.265625" collapsed="true"/>
+    <col min="6" max="6" style="1" width="9.19921875" collapsed="true"/>
+    <col min="7" max="7" customWidth="true" style="1" width="14.19921875" collapsed="true"/>
+    <col min="8" max="16384" style="1" width="9.19921875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4164,12 +4493,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>184</v>
+        <v>325</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>32</v>
@@ -4181,18 +4510,18 @@
         <v>17</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>113</v>
+        <v>127</v>
       </c>
       <c r="G2" s="1" t="s">
         <v>93</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>35</v>
       </c>
       <c r="B3" t="s">
-        <v>185</v>
+        <v>326</v>
       </c>
       <c r="C3" s="1" t="s">
         <v>32</v>
@@ -4204,18 +4533,18 @@
         <v>17</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="G3" s="1" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>186</v>
+        <v>327</v>
       </c>
       <c r="C4" s="1" t="s">
         <v>32</v>
@@ -4227,18 +4556,18 @@
         <v>17</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>37</v>
+        <v>113</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>35</v>
       </c>
       <c r="B5" t="s">
-        <v>187</v>
+        <v>328</v>
       </c>
       <c r="C5" s="1" t="s">
         <v>32</v>
@@ -4250,18 +4579,18 @@
         <v>17</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="G5" s="1" t="s">
         <v>94</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>35</v>
       </c>
       <c r="B6" t="s">
-        <v>188</v>
+        <v>329</v>
       </c>
       <c r="C6" s="1" t="s">
         <v>32</v>
@@ -4273,7 +4602,7 @@
         <v>17</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>30</v>
+        <v>18</v>
       </c>
       <c r="G6" s="1" t="s">
         <v>94</v>
@@ -4287,17 +4616,17 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{03F3D31C-4F04-42F4-8C54-828F1948951D}">
   <dimension ref="A1:G3"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.19921875" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" style="1" width="9.1796875" collapsed="true"/>
-    <col min="2" max="2" customWidth="true" style="1" width="32.453125" collapsed="true"/>
-    <col min="3" max="3" customWidth="true" style="1" width="16.7265625" collapsed="true"/>
-    <col min="4" max="4" customWidth="true" style="1" width="50.81640625" collapsed="true"/>
-    <col min="5" max="5" customWidth="true" style="1" width="46.26953125" collapsed="true"/>
-    <col min="6" max="16384" style="1" width="9.1796875" collapsed="true"/>
+    <col min="1" max="1" style="1" width="9.19921875" collapsed="true"/>
+    <col min="2" max="2" customWidth="true" style="1" width="32.46484375" collapsed="true"/>
+    <col min="3" max="3" customWidth="true" style="1" width="16.73046875" collapsed="true"/>
+    <col min="4" max="4" customWidth="true" style="1" width="50.796875" collapsed="true"/>
+    <col min="5" max="5" customWidth="true" style="1" width="46.265625" collapsed="true"/>
+    <col min="6" max="16384" style="1" width="9.19921875" collapsed="true"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -4317,12 +4646,12 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>35</v>
       </c>
       <c r="B2" t="s">
-        <v>178</v>
+        <v>319</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>32</v>
@@ -4337,7 +4666,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>35</v>
       </c>

</xml_diff>